<commit_message>
:construction: Codes and programs
I added the codes for orhogonalizing the shocks and added the input for omputing the local projections
</commit_message>
<xml_diff>
--- a/Monetary Policy Shocks/Series_ChoquesPM_JVROMERO.xlsx
+++ b/Monetary Policy Shocks/Series_ChoquesPM_JVROMERO.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://bancodelarepublica-my.sharepoint.com/personal/jromerch_banrep_gov_co/Documents/Desktop/03_MY RESEARCH/CHOQUES DE PM/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Disco C\Repositorios Git\Monetary-Policy-Shocks-and-Central-bank-information-in-Colombia\Monetary Policy Shocks\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="277" documentId="8_{523CFCB0-19FA-45EC-B4C2-84D38A8F36FF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9B9BF870-5639-4681-9830-1CC96F7FE368}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A07CE190-85E7-48E4-AC58-DCFB3E66ECCD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="1740" windowWidth="20730" windowHeight="11040" xr2:uid="{09EFE9E4-A311-420D-BE74-8BB279DD0F97}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{09EFE9E4-A311-420D-BE74-8BB279DD0F97}"/>
   </bookViews>
   <sheets>
     <sheet name="MPShocks_DESDE2008" sheetId="1" r:id="rId1"/>
@@ -111,8 +111,8 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
-    <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
-    <numFmt numFmtId="164" formatCode="0.000"/>
+    <numFmt numFmtId="164" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="165" formatCode="0.000"/>
   </numFmts>
   <fonts count="9" x14ac:knownFonts="1">
     <font>
@@ -302,7 +302,7 @@
   </borders>
   <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
   <cellXfs count="22">
@@ -324,14 +324,14 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="17" fontId="8" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="164" fontId="3" fillId="2" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="164" fontId="3" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="165" fontId="3" fillId="2" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="165" fontId="3" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="9" fontId="6" fillId="2" borderId="3" xfId="2" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="43" fontId="8" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="164" fontId="8" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="2" fontId="8" fillId="2" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="43" fontId="3" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="164" fontId="3" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Millares" xfId="1" builtinId="3"/>
@@ -7024,10 +7024,6 @@
 </xdr:wsDr>
 </file>
 
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - Tema de 2022">
   <a:themeElements>
@@ -7326,23 +7322,23 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FC732F9A-CB73-42D8-A101-2C99F85D81B8}">
   <dimension ref="A1:J217"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.44140625" defaultRowHeight="15.6" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="15.5703125" style="2" customWidth="1"/>
-    <col min="2" max="2" width="50.28515625" style="2" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="15.5546875" style="2" customWidth="1"/>
+    <col min="2" max="2" width="50.33203125" style="2" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="30" style="2" customWidth="1"/>
-    <col min="4" max="16384" width="11.42578125" style="2"/>
+    <col min="4" max="16384" width="11.44140625" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:10" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:10" ht="16.2" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A2" s="1"/>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A3" s="3" t="s">
         <v>6</v>
       </c>
@@ -7356,7 +7352,7 @@
       <c r="I3" s="4"/>
       <c r="J3" s="5"/>
     </row>
-    <row r="4" spans="1:10" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:10" ht="17.399999999999999" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A4" s="6" t="s">
         <v>7</v>
       </c>
@@ -7370,10 +7366,10 @@
       <c r="I4" s="7"/>
       <c r="J4" s="8"/>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A5" s="9"/>
     </row>
-    <row r="6" spans="1:10" ht="39.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:10" ht="39.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="10" t="s">
         <v>5</v>
       </c>
@@ -7384,7 +7380,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="7" spans="1:10" ht="17.25" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A7" s="12" t="s">
         <v>0</v>
       </c>
@@ -7395,7 +7391,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A8" s="13">
         <v>39472</v>
       </c>
@@ -7407,7 +7403,7 @@
       </c>
       <c r="E8" s="15"/>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A9" s="13">
         <v>39500</v>
       </c>
@@ -7419,7 +7415,7 @@
       </c>
       <c r="E9" s="15"/>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A10" s="13">
         <v>39535</v>
       </c>
@@ -7431,7 +7427,7 @@
       </c>
       <c r="E10" s="15"/>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A11" s="13">
         <v>39563</v>
       </c>
@@ -7443,7 +7439,7 @@
       </c>
       <c r="E11" s="15"/>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A12" s="13">
         <v>39591</v>
       </c>
@@ -7455,7 +7451,7 @@
       </c>
       <c r="E12" s="15"/>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A13" s="13">
         <v>39619</v>
       </c>
@@ -7467,7 +7463,7 @@
       </c>
       <c r="E13" s="15"/>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A14" s="13">
         <v>39654</v>
       </c>
@@ -7479,7 +7475,7 @@
       </c>
       <c r="E14" s="15"/>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A15" s="13">
         <v>39675</v>
       </c>
@@ -7491,7 +7487,7 @@
       </c>
       <c r="E15" s="15"/>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A16" s="13">
         <v>39710</v>
       </c>
@@ -7503,7 +7499,7 @@
       </c>
       <c r="E16" s="15"/>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A17" s="13">
         <v>39745</v>
       </c>
@@ -7515,7 +7511,7 @@
       </c>
       <c r="E17" s="15"/>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A18" s="13">
         <v>39773</v>
       </c>
@@ -7527,7 +7523,7 @@
       </c>
       <c r="E18" s="15"/>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A19" s="13">
         <v>39801</v>
       </c>
@@ -7539,7 +7535,7 @@
       </c>
       <c r="E19" s="15"/>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A20" s="13">
         <v>39843</v>
       </c>
@@ -7551,7 +7547,7 @@
       </c>
       <c r="E20" s="15"/>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A21" s="13">
         <v>39871</v>
       </c>
@@ -7563,7 +7559,7 @@
       </c>
       <c r="E21" s="15"/>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A22" s="13">
         <v>39892</v>
       </c>
@@ -7575,7 +7571,7 @@
       </c>
       <c r="E22" s="15"/>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A23" s="13">
         <v>39933</v>
       </c>
@@ -7587,7 +7583,7 @@
       </c>
       <c r="E23" s="15"/>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A24" s="13">
         <v>39962</v>
       </c>
@@ -7599,7 +7595,7 @@
       </c>
       <c r="E24" s="15"/>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A25" s="13">
         <v>39983</v>
       </c>
@@ -7611,7 +7607,7 @@
       </c>
       <c r="E25" s="15"/>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A26" s="13">
         <v>40018</v>
       </c>
@@ -7623,7 +7619,7 @@
       </c>
       <c r="E26" s="15"/>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A27" s="13">
         <v>40053</v>
       </c>
@@ -7635,7 +7631,7 @@
       </c>
       <c r="E27" s="15"/>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A28" s="13">
         <v>40081</v>
       </c>
@@ -7647,7 +7643,7 @@
       </c>
       <c r="E28" s="15"/>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A29" s="13">
         <v>40109</v>
       </c>
@@ -7659,7 +7655,7 @@
       </c>
       <c r="E29" s="15"/>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A30" s="13">
         <v>40137</v>
       </c>
@@ -7671,7 +7667,7 @@
       </c>
       <c r="E30" s="15"/>
     </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A31" s="13">
         <v>40165</v>
       </c>
@@ -7683,7 +7679,7 @@
       </c>
       <c r="E31" s="15"/>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A32" s="13">
         <v>40207</v>
       </c>
@@ -7695,7 +7691,7 @@
       </c>
       <c r="E32" s="15"/>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A33" s="13">
         <v>40235</v>
       </c>
@@ -7707,7 +7703,7 @@
       </c>
       <c r="E33" s="15"/>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A34" s="13">
         <v>40263</v>
       </c>
@@ -7719,7 +7715,7 @@
       </c>
       <c r="E34" s="15"/>
     </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A35" s="13">
         <v>40298</v>
       </c>
@@ -7731,7 +7727,7 @@
       </c>
       <c r="E35" s="15"/>
     </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A36" s="13">
         <v>40325</v>
       </c>
@@ -7743,7 +7739,7 @@
       </c>
       <c r="E36" s="15"/>
     </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A37" s="13">
         <v>40347</v>
       </c>
@@ -7755,7 +7751,7 @@
       </c>
       <c r="E37" s="15"/>
     </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A38" s="13">
         <v>40382</v>
       </c>
@@ -7767,7 +7763,7 @@
       </c>
       <c r="E38" s="15"/>
     </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A39" s="13">
         <v>40410</v>
       </c>
@@ -7779,7 +7775,7 @@
       </c>
       <c r="E39" s="15"/>
     </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A40" s="13">
         <v>40445</v>
       </c>
@@ -7791,7 +7787,7 @@
       </c>
       <c r="E40" s="15"/>
     </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A41" s="13">
         <v>40480</v>
       </c>
@@ -7803,7 +7799,7 @@
       </c>
       <c r="E41" s="15"/>
     </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A42" s="13">
         <v>40501</v>
       </c>
@@ -7815,7 +7811,7 @@
       </c>
       <c r="E42" s="15"/>
     </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A43" s="13">
         <v>40529</v>
       </c>
@@ -7827,7 +7823,7 @@
       </c>
       <c r="E43" s="15"/>
     </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A44" s="13">
         <v>40574</v>
       </c>
@@ -7839,7 +7835,7 @@
       </c>
       <c r="E44" s="15"/>
     </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A45" s="13">
         <v>40599</v>
       </c>
@@ -7851,7 +7847,7 @@
       </c>
       <c r="E45" s="15"/>
     </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A46" s="13">
         <v>40620</v>
       </c>
@@ -7863,7 +7859,7 @@
       </c>
       <c r="E46" s="15"/>
     </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A47" s="13">
         <v>40662</v>
       </c>
@@ -7875,7 +7871,7 @@
       </c>
       <c r="E47" s="15"/>
     </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A48" s="13">
         <v>40693</v>
       </c>
@@ -7887,7 +7883,7 @@
       </c>
       <c r="E48" s="15"/>
     </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A49" s="13">
         <v>40711</v>
       </c>
@@ -7899,7 +7895,7 @@
       </c>
       <c r="E49" s="15"/>
     </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A50" s="13">
         <v>40753</v>
       </c>
@@ -7911,7 +7907,7 @@
       </c>
       <c r="E50" s="15"/>
     </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A51" s="13">
         <v>40774</v>
       </c>
@@ -7923,7 +7919,7 @@
       </c>
       <c r="E51" s="15"/>
     </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A52" s="13">
         <v>40816</v>
       </c>
@@ -7935,7 +7931,7 @@
       </c>
       <c r="E52" s="15"/>
     </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A53" s="13">
         <v>40844</v>
       </c>
@@ -7947,7 +7943,7 @@
       </c>
       <c r="E53" s="15"/>
     </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A54" s="13">
         <v>40872</v>
       </c>
@@ -7959,7 +7955,7 @@
       </c>
       <c r="E54" s="15"/>
     </row>
-    <row r="55" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A55" s="13">
         <v>40893</v>
       </c>
@@ -7971,7 +7967,7 @@
       </c>
       <c r="E55" s="15"/>
     </row>
-    <row r="56" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A56" s="13">
         <v>40938</v>
       </c>
@@ -7983,7 +7979,7 @@
       </c>
       <c r="E56" s="15"/>
     </row>
-    <row r="57" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A57" s="13">
         <v>40963</v>
       </c>
@@ -7995,7 +7991,7 @@
       </c>
       <c r="E57" s="15"/>
     </row>
-    <row r="58" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A58" s="13">
         <v>40991</v>
       </c>
@@ -8007,7 +8003,7 @@
       </c>
       <c r="E58" s="15"/>
     </row>
-    <row r="59" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A59" s="13">
         <v>41029</v>
       </c>
@@ -8019,7 +8015,7 @@
       </c>
       <c r="E59" s="15"/>
     </row>
-    <row r="60" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A60" s="13">
         <v>41057</v>
       </c>
@@ -8031,7 +8027,7 @@
       </c>
       <c r="E60" s="15"/>
     </row>
-    <row r="61" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A61" s="13">
         <v>41089</v>
       </c>
@@ -8043,7 +8039,7 @@
       </c>
       <c r="E61" s="15"/>
     </row>
-    <row r="62" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A62" s="13">
         <v>41117</v>
       </c>
@@ -8055,7 +8051,7 @@
       </c>
       <c r="E62" s="15"/>
     </row>
-    <row r="63" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A63" s="13">
         <v>41145</v>
       </c>
@@ -8067,7 +8063,7 @@
       </c>
       <c r="E63" s="15"/>
     </row>
-    <row r="64" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A64" s="13">
         <v>41180</v>
       </c>
@@ -8079,7 +8075,7 @@
       </c>
       <c r="E64" s="15"/>
     </row>
-    <row r="65" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A65" s="13">
         <v>41208</v>
       </c>
@@ -8091,7 +8087,7 @@
       </c>
       <c r="E65" s="15"/>
     </row>
-    <row r="66" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A66" s="13">
         <v>41236</v>
       </c>
@@ -8103,7 +8099,7 @@
       </c>
       <c r="E66" s="15"/>
     </row>
-    <row r="67" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A67" s="13">
         <v>41264</v>
       </c>
@@ -8115,7 +8111,7 @@
       </c>
       <c r="E67" s="15"/>
     </row>
-    <row r="68" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A68" s="13">
         <v>41302</v>
       </c>
@@ -8127,7 +8123,7 @@
       </c>
       <c r="E68" s="15"/>
     </row>
-    <row r="69" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A69" s="13">
         <v>41327</v>
       </c>
@@ -8139,7 +8135,7 @@
       </c>
       <c r="E69" s="15"/>
     </row>
-    <row r="70" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A70" s="13">
         <v>41355</v>
       </c>
@@ -8151,7 +8147,7 @@
       </c>
       <c r="E70" s="15"/>
     </row>
-    <row r="71" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A71" s="13">
         <v>41390</v>
       </c>
@@ -8163,7 +8159,7 @@
       </c>
       <c r="E71" s="15"/>
     </row>
-    <row r="72" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A72" s="13">
         <v>41425</v>
       </c>
@@ -8175,7 +8171,7 @@
       </c>
       <c r="E72" s="15"/>
     </row>
-    <row r="73" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A73" s="13">
         <v>41453</v>
       </c>
@@ -8187,7 +8183,7 @@
       </c>
       <c r="E73" s="15"/>
     </row>
-    <row r="74" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A74" s="13">
         <v>41481</v>
       </c>
@@ -8199,7 +8195,7 @@
       </c>
       <c r="E74" s="15"/>
     </row>
-    <row r="75" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A75" s="13">
         <v>41516</v>
       </c>
@@ -8211,7 +8207,7 @@
       </c>
       <c r="E75" s="15"/>
     </row>
-    <row r="76" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A76" s="13">
         <v>41544</v>
       </c>
@@ -8223,7 +8219,7 @@
       </c>
       <c r="E76" s="15"/>
     </row>
-    <row r="77" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A77" s="13">
         <v>41572</v>
       </c>
@@ -8235,7 +8231,7 @@
       </c>
       <c r="E77" s="15"/>
     </row>
-    <row r="78" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A78" s="13">
         <v>41607</v>
       </c>
@@ -8247,7 +8243,7 @@
       </c>
       <c r="E78" s="15"/>
     </row>
-    <row r="79" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A79" s="13">
         <v>41628</v>
       </c>
@@ -8259,7 +8255,7 @@
       </c>
       <c r="E79" s="15"/>
     </row>
-    <row r="80" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A80" s="13">
         <v>41670</v>
       </c>
@@ -8271,7 +8267,7 @@
       </c>
       <c r="E80" s="15"/>
     </row>
-    <row r="81" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A81" s="13">
         <v>41698</v>
       </c>
@@ -8283,7 +8279,7 @@
       </c>
       <c r="E81" s="15"/>
     </row>
-    <row r="82" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A82" s="13">
         <v>41719</v>
       </c>
@@ -8295,7 +8291,7 @@
       </c>
       <c r="E82" s="15"/>
     </row>
-    <row r="83" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A83" s="13">
         <v>41754</v>
       </c>
@@ -8307,7 +8303,7 @@
       </c>
       <c r="E83" s="15"/>
     </row>
-    <row r="84" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A84" s="13">
         <v>41789</v>
       </c>
@@ -8319,7 +8315,7 @@
       </c>
       <c r="E84" s="15"/>
     </row>
-    <row r="85" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A85" s="13">
         <v>41810</v>
       </c>
@@ -8331,7 +8327,7 @@
       </c>
       <c r="E85" s="15"/>
     </row>
-    <row r="86" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A86" s="13">
         <v>41851</v>
       </c>
@@ -8343,7 +8339,7 @@
       </c>
       <c r="E86" s="15"/>
     </row>
-    <row r="87" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A87" s="13">
         <v>41880</v>
       </c>
@@ -8355,7 +8351,7 @@
       </c>
       <c r="E87" s="15"/>
     </row>
-    <row r="88" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A88" s="13">
         <v>41908</v>
       </c>
@@ -8367,7 +8363,7 @@
       </c>
       <c r="E88" s="15"/>
     </row>
-    <row r="89" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A89" s="13">
         <v>41942</v>
       </c>
@@ -8379,7 +8375,7 @@
       </c>
       <c r="E89" s="15"/>
     </row>
-    <row r="90" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A90" s="13">
         <v>41971</v>
       </c>
@@ -8391,7 +8387,7 @@
       </c>
       <c r="E90" s="15"/>
     </row>
-    <row r="91" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A91" s="13">
         <v>41992</v>
       </c>
@@ -8403,7 +8399,7 @@
       </c>
       <c r="E91" s="15"/>
     </row>
-    <row r="92" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A92" s="13">
         <v>42034</v>
       </c>
@@ -8415,7 +8411,7 @@
       </c>
       <c r="E92" s="15"/>
     </row>
-    <row r="93" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A93" s="13">
         <v>42055</v>
       </c>
@@ -8427,7 +8423,7 @@
       </c>
       <c r="E93" s="15"/>
     </row>
-    <row r="94" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A94" s="13">
         <v>42083</v>
       </c>
@@ -8439,7 +8435,7 @@
       </c>
       <c r="E94" s="15"/>
     </row>
-    <row r="95" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A95" s="13">
         <v>42118</v>
       </c>
@@ -8451,7 +8447,7 @@
       </c>
       <c r="E95" s="15"/>
     </row>
-    <row r="96" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A96" s="13">
         <v>42146</v>
       </c>
@@ -8463,7 +8459,7 @@
       </c>
       <c r="E96" s="15"/>
     </row>
-    <row r="97" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A97" s="13">
         <v>42179</v>
       </c>
@@ -8475,7 +8471,7 @@
       </c>
       <c r="E97" s="15"/>
     </row>
-    <row r="98" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A98" s="13">
         <v>42216</v>
       </c>
@@ -8487,7 +8483,7 @@
       </c>
       <c r="E98" s="15"/>
     </row>
-    <row r="99" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A99" s="13">
         <v>42237</v>
       </c>
@@ -8499,7 +8495,7 @@
       </c>
       <c r="E99" s="15"/>
     </row>
-    <row r="100" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A100" s="13">
         <v>42272</v>
       </c>
@@ -8511,7 +8507,7 @@
       </c>
       <c r="E100" s="15"/>
     </row>
-    <row r="101" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A101" s="13">
         <v>42307</v>
       </c>
@@ -8523,7 +8519,7 @@
       </c>
       <c r="E101" s="15"/>
     </row>
-    <row r="102" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A102" s="13">
         <v>42335</v>
       </c>
@@ -8535,7 +8531,7 @@
       </c>
       <c r="E102" s="15"/>
     </row>
-    <row r="103" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A103" s="13">
         <v>42356</v>
       </c>
@@ -8547,7 +8543,7 @@
       </c>
       <c r="E103" s="15"/>
     </row>
-    <row r="104" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A104" s="13">
         <v>42398</v>
       </c>
@@ -8559,7 +8555,7 @@
       </c>
       <c r="E104" s="15"/>
     </row>
-    <row r="105" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A105" s="13">
         <v>42419</v>
       </c>
@@ -8571,7 +8567,7 @@
       </c>
       <c r="E105" s="15"/>
     </row>
-    <row r="106" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A106" s="13">
         <v>42447</v>
       </c>
@@ -8583,7 +8579,7 @@
       </c>
       <c r="E106" s="15"/>
     </row>
-    <row r="107" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A107" s="13">
         <v>42489</v>
       </c>
@@ -8595,7 +8591,7 @@
       </c>
       <c r="E107" s="15"/>
     </row>
-    <row r="108" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A108" s="13">
         <v>42517</v>
       </c>
@@ -8607,7 +8603,7 @@
       </c>
       <c r="E108" s="15"/>
     </row>
-    <row r="109" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A109" s="13">
         <v>42543</v>
       </c>
@@ -8619,7 +8615,7 @@
       </c>
       <c r="E109" s="15"/>
     </row>
-    <row r="110" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A110" s="13">
         <v>42580</v>
       </c>
@@ -8631,7 +8627,7 @@
       </c>
       <c r="E110" s="15"/>
     </row>
-    <row r="111" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A111" s="13">
         <v>42613</v>
       </c>
@@ -8643,7 +8639,7 @@
       </c>
       <c r="E111" s="15"/>
     </row>
-    <row r="112" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A112" s="13">
         <v>42643</v>
       </c>
@@ -8655,7 +8651,7 @@
       </c>
       <c r="E112" s="15"/>
     </row>
-    <row r="113" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="113" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A113" s="13">
         <v>42671</v>
       </c>
@@ -8667,7 +8663,7 @@
       </c>
       <c r="E113" s="15"/>
     </row>
-    <row r="114" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="114" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A114" s="13">
         <v>42699</v>
       </c>
@@ -8679,7 +8675,7 @@
       </c>
       <c r="E114" s="15"/>
     </row>
-    <row r="115" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A115" s="13">
         <v>42720</v>
       </c>
@@ -8691,7 +8687,7 @@
       </c>
       <c r="E115" s="15"/>
     </row>
-    <row r="116" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="116" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A116" s="13">
         <v>42762</v>
       </c>
@@ -8703,7 +8699,7 @@
       </c>
       <c r="E116" s="15"/>
     </row>
-    <row r="117" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="117" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A117" s="13">
         <v>42790</v>
       </c>
@@ -8715,7 +8711,7 @@
       </c>
       <c r="E117" s="15"/>
     </row>
-    <row r="118" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="118" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A118" s="13">
         <v>42818</v>
       </c>
@@ -8727,7 +8723,7 @@
       </c>
       <c r="E118" s="15"/>
     </row>
-    <row r="119" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="119" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A119" s="13">
         <v>42853</v>
       </c>
@@ -8739,7 +8735,7 @@
       </c>
       <c r="E119" s="15"/>
     </row>
-    <row r="120" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="120" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A120" s="13">
         <v>42881</v>
       </c>
@@ -8751,7 +8747,7 @@
       </c>
       <c r="E120" s="15"/>
     </row>
-    <row r="121" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="121" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A121" s="13">
         <v>42916</v>
       </c>
@@ -8763,7 +8759,7 @@
       </c>
       <c r="E121" s="15"/>
     </row>
-    <row r="122" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="122" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A122" s="13">
         <v>42943</v>
       </c>
@@ -8775,7 +8771,7 @@
       </c>
       <c r="E122" s="15"/>
     </row>
-    <row r="123" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="123" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A123" s="13">
         <v>42978</v>
       </c>
@@ -8787,7 +8783,7 @@
       </c>
       <c r="E123" s="15"/>
     </row>
-    <row r="124" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="124" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A124" s="13">
         <v>43007</v>
       </c>
@@ -8799,7 +8795,7 @@
       </c>
       <c r="E124" s="15"/>
     </row>
-    <row r="125" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="125" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A125" s="13">
         <v>43035</v>
       </c>
@@ -8811,7 +8807,7 @@
       </c>
       <c r="E125" s="15"/>
     </row>
-    <row r="126" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="126" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A126" s="13">
         <v>43063</v>
       </c>
@@ -8823,7 +8819,7 @@
       </c>
       <c r="E126" s="15"/>
     </row>
-    <row r="127" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="127" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A127" s="13">
         <v>43083</v>
       </c>
@@ -8835,7 +8831,7 @@
       </c>
       <c r="E127" s="15"/>
     </row>
-    <row r="128" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="128" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A128" s="13">
         <v>43129</v>
       </c>
@@ -8847,7 +8843,7 @@
       </c>
       <c r="E128" s="15"/>
     </row>
-    <row r="129" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="129" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A129" s="13">
         <v>43132</v>
       </c>
@@ -8859,7 +8855,7 @@
       </c>
       <c r="E129" s="15"/>
     </row>
-    <row r="130" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="130" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A130" s="13">
         <v>43179</v>
       </c>
@@ -8871,7 +8867,7 @@
       </c>
       <c r="E130" s="15"/>
     </row>
-    <row r="131" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="131" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A131" s="13">
         <v>43217</v>
       </c>
@@ -8883,7 +8879,7 @@
       </c>
       <c r="E131" s="15"/>
     </row>
-    <row r="132" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="132" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A132" s="13">
         <v>43221</v>
       </c>
@@ -8895,7 +8891,7 @@
       </c>
       <c r="E132" s="15"/>
     </row>
-    <row r="133" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="133" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A133" s="13">
         <v>43280</v>
       </c>
@@ -8907,7 +8903,7 @@
       </c>
       <c r="E133" s="15"/>
     </row>
-    <row r="134" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="134" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A134" s="13">
         <v>43308</v>
       </c>
@@ -8919,7 +8915,7 @@
       </c>
       <c r="E134" s="15"/>
     </row>
-    <row r="135" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="135" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A135" s="13">
         <v>43313</v>
       </c>
@@ -8931,7 +8927,7 @@
       </c>
       <c r="E135" s="15"/>
     </row>
-    <row r="136" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="136" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A136" s="13">
         <v>43371</v>
       </c>
@@ -8943,7 +8939,7 @@
       </c>
       <c r="E136" s="15"/>
     </row>
-    <row r="137" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="137" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A137" s="13">
         <v>43399</v>
       </c>
@@ -8955,7 +8951,7 @@
       </c>
       <c r="E137" s="15"/>
     </row>
-    <row r="138" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="138" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A138" s="13">
         <v>43405</v>
       </c>
@@ -8967,7 +8963,7 @@
       </c>
       <c r="E138" s="15"/>
     </row>
-    <row r="139" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="139" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A139" s="13">
         <v>43455</v>
       </c>
@@ -8979,7 +8975,7 @@
       </c>
       <c r="E139" s="15"/>
     </row>
-    <row r="140" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="140" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A140" s="13">
         <v>43496</v>
       </c>
@@ -8991,7 +8987,7 @@
       </c>
       <c r="E140" s="15"/>
     </row>
-    <row r="141" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="141" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A141" s="13">
         <v>43497</v>
       </c>
@@ -9003,7 +8999,7 @@
       </c>
       <c r="E141" s="15"/>
     </row>
-    <row r="142" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="142" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A142" s="13">
         <v>43546</v>
       </c>
@@ -9015,7 +9011,7 @@
       </c>
       <c r="E142" s="15"/>
     </row>
-    <row r="143" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="143" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A143" s="13">
         <v>43581</v>
       </c>
@@ -9027,7 +9023,7 @@
       </c>
       <c r="E143" s="15"/>
     </row>
-    <row r="144" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="144" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A144" s="13">
         <v>43586</v>
       </c>
@@ -9039,7 +9035,7 @@
       </c>
       <c r="E144" s="15"/>
     </row>
-    <row r="145" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="145" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A145" s="13">
         <v>43637</v>
       </c>
@@ -9051,7 +9047,7 @@
       </c>
       <c r="E145" s="15"/>
     </row>
-    <row r="146" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="146" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A146" s="13">
         <v>43672</v>
       </c>
@@ -9063,7 +9059,7 @@
       </c>
       <c r="E146" s="15"/>
     </row>
-    <row r="147" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="147" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A147" s="13">
         <v>43678</v>
       </c>
@@ -9075,7 +9071,7 @@
       </c>
       <c r="E147" s="15"/>
     </row>
-    <row r="148" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="148" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A148" s="13">
         <v>43731</v>
       </c>
@@ -9087,7 +9083,7 @@
       </c>
       <c r="E148" s="15"/>
     </row>
-    <row r="149" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="149" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A149" s="13">
         <v>43769</v>
       </c>
@@ -9099,7 +9095,7 @@
       </c>
       <c r="E149" s="15"/>
     </row>
-    <row r="150" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="150" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A150" s="13">
         <v>43770</v>
       </c>
@@ -9111,7 +9107,7 @@
       </c>
       <c r="E150" s="15"/>
     </row>
-    <row r="151" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="151" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A151" s="13">
         <v>43800</v>
       </c>
@@ -9123,7 +9119,7 @@
       </c>
       <c r="E151" s="15"/>
     </row>
-    <row r="152" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="152" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A152" s="13">
         <v>43831</v>
       </c>
@@ -9135,7 +9131,7 @@
       </c>
       <c r="E152" s="15"/>
     </row>
-    <row r="153" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="153" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A153" s="13">
         <v>43862</v>
       </c>
@@ -9147,7 +9143,7 @@
       </c>
       <c r="E153" s="15"/>
     </row>
-    <row r="154" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="154" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A154" s="13">
         <v>43891</v>
       </c>
@@ -9159,7 +9155,7 @@
       </c>
       <c r="E154" s="15"/>
     </row>
-    <row r="155" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="155" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A155" s="13">
         <v>43922</v>
       </c>
@@ -9171,7 +9167,7 @@
       </c>
       <c r="E155" s="15"/>
     </row>
-    <row r="156" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="156" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A156" s="13">
         <v>43952</v>
       </c>
@@ -9183,7 +9179,7 @@
       </c>
       <c r="E156" s="15"/>
     </row>
-    <row r="157" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="157" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A157" s="13">
         <v>43983</v>
       </c>
@@ -9195,7 +9191,7 @@
       </c>
       <c r="E157" s="15"/>
     </row>
-    <row r="158" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="158" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A158" s="13">
         <v>44013</v>
       </c>
@@ -9207,7 +9203,7 @@
       </c>
       <c r="E158" s="15"/>
     </row>
-    <row r="159" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="159" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A159" s="13">
         <v>44044</v>
       </c>
@@ -9219,7 +9215,7 @@
       </c>
       <c r="E159" s="15"/>
     </row>
-    <row r="160" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="160" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A160" s="13">
         <v>44075</v>
       </c>
@@ -9231,7 +9227,7 @@
       </c>
       <c r="E160" s="15"/>
     </row>
-    <row r="161" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="161" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A161" s="13">
         <v>44105</v>
       </c>
@@ -9243,7 +9239,7 @@
       </c>
       <c r="E161" s="15"/>
     </row>
-    <row r="162" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="162" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A162" s="13">
         <v>44136</v>
       </c>
@@ -9255,7 +9251,7 @@
       </c>
       <c r="E162" s="15"/>
     </row>
-    <row r="163" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="163" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A163" s="13">
         <v>44166</v>
       </c>
@@ -9267,7 +9263,7 @@
       </c>
       <c r="E163" s="15"/>
     </row>
-    <row r="164" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="164" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A164" s="13">
         <v>44197</v>
       </c>
@@ -9279,7 +9275,7 @@
       </c>
       <c r="E164" s="15"/>
     </row>
-    <row r="165" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="165" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A165" s="13">
         <v>44228</v>
       </c>
@@ -9291,7 +9287,7 @@
       </c>
       <c r="E165" s="15"/>
     </row>
-    <row r="166" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="166" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A166" s="13">
         <v>44256</v>
       </c>
@@ -9303,7 +9299,7 @@
       </c>
       <c r="E166" s="15"/>
     </row>
-    <row r="167" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="167" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A167" s="13">
         <v>44287</v>
       </c>
@@ -9315,7 +9311,7 @@
       </c>
       <c r="E167" s="15"/>
     </row>
-    <row r="168" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="168" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A168" s="13">
         <v>44317</v>
       </c>
@@ -9327,7 +9323,7 @@
       </c>
       <c r="E168" s="15"/>
     </row>
-    <row r="169" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="169" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A169" s="13">
         <v>44348</v>
       </c>
@@ -9339,7 +9335,7 @@
       </c>
       <c r="E169" s="15"/>
     </row>
-    <row r="170" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="170" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A170" s="13">
         <v>44378</v>
       </c>
@@ -9351,7 +9347,7 @@
       </c>
       <c r="E170" s="15"/>
     </row>
-    <row r="171" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="171" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A171" s="13">
         <v>44409</v>
       </c>
@@ -9363,7 +9359,7 @@
       </c>
       <c r="E171" s="15"/>
     </row>
-    <row r="172" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="172" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A172" s="13">
         <v>44440</v>
       </c>
@@ -9375,7 +9371,7 @@
       </c>
       <c r="E172" s="15"/>
     </row>
-    <row r="173" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="173" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A173" s="13">
         <v>44470</v>
       </c>
@@ -9387,7 +9383,7 @@
       </c>
       <c r="E173" s="15"/>
     </row>
-    <row r="174" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="174" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A174" s="13">
         <v>44501</v>
       </c>
@@ -9399,7 +9395,7 @@
       </c>
       <c r="E174" s="15"/>
     </row>
-    <row r="175" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="175" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A175" s="13">
         <v>44531</v>
       </c>
@@ -9411,7 +9407,7 @@
       </c>
       <c r="E175" s="15"/>
     </row>
-    <row r="176" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="176" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A176" s="13">
         <v>44562</v>
       </c>
@@ -9423,7 +9419,7 @@
       </c>
       <c r="E176" s="15"/>
     </row>
-    <row r="177" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="177" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A177" s="13">
         <v>44593</v>
       </c>
@@ -9435,7 +9431,7 @@
       </c>
       <c r="E177" s="15"/>
     </row>
-    <row r="178" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="178" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A178" s="13">
         <v>44621</v>
       </c>
@@ -9447,7 +9443,7 @@
       </c>
       <c r="E178" s="15"/>
     </row>
-    <row r="179" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="179" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A179" s="13">
         <v>44652</v>
       </c>
@@ -9459,7 +9455,7 @@
       </c>
       <c r="E179" s="15"/>
     </row>
-    <row r="180" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="180" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A180" s="13">
         <v>44682</v>
       </c>
@@ -9471,7 +9467,7 @@
       </c>
       <c r="E180" s="15"/>
     </row>
-    <row r="181" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="181" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A181" s="13">
         <v>44713</v>
       </c>
@@ -9483,7 +9479,7 @@
       </c>
       <c r="E181" s="15"/>
     </row>
-    <row r="182" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="182" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A182" s="13">
         <v>44743</v>
       </c>
@@ -9495,7 +9491,7 @@
       </c>
       <c r="E182" s="15"/>
     </row>
-    <row r="183" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="183" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A183" s="13">
         <v>44774</v>
       </c>
@@ -9507,7 +9503,7 @@
       </c>
       <c r="E183" s="15"/>
     </row>
-    <row r="184" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="184" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A184" s="13">
         <v>44805</v>
       </c>
@@ -9519,7 +9515,7 @@
       </c>
       <c r="E184" s="15"/>
     </row>
-    <row r="185" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="185" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A185" s="13">
         <v>44835</v>
       </c>
@@ -9531,7 +9527,7 @@
       </c>
       <c r="E185" s="15"/>
     </row>
-    <row r="186" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="186" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A186" s="13">
         <v>44866</v>
       </c>
@@ -9543,7 +9539,7 @@
       </c>
       <c r="E186" s="15"/>
     </row>
-    <row r="187" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="187" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A187" s="13">
         <v>44896</v>
       </c>
@@ -9555,7 +9551,7 @@
       </c>
       <c r="E187" s="15"/>
     </row>
-    <row r="188" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="188" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A188" s="13">
         <v>44927</v>
       </c>
@@ -9567,7 +9563,7 @@
       </c>
       <c r="E188" s="15"/>
     </row>
-    <row r="189" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="189" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A189" s="13">
         <v>44958</v>
       </c>
@@ -9579,7 +9575,7 @@
       </c>
       <c r="E189" s="15"/>
     </row>
-    <row r="190" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="190" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A190" s="13">
         <v>44986</v>
       </c>
@@ -9591,7 +9587,7 @@
       </c>
       <c r="E190" s="15"/>
     </row>
-    <row r="191" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="191" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A191" s="13">
         <v>45017</v>
       </c>
@@ -9603,7 +9599,7 @@
       </c>
       <c r="E191" s="15"/>
     </row>
-    <row r="192" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="192" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A192" s="13">
         <v>45047</v>
       </c>
@@ -9615,7 +9611,7 @@
       </c>
       <c r="E192" s="15"/>
     </row>
-    <row r="193" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="193" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A193" s="13">
         <v>45078</v>
       </c>
@@ -9627,7 +9623,7 @@
       </c>
       <c r="E193" s="15"/>
     </row>
-    <row r="194" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="194" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A194" s="13">
         <v>45108</v>
       </c>
@@ -9639,7 +9635,7 @@
       </c>
       <c r="E194" s="15"/>
     </row>
-    <row r="195" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="195" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A195" s="13">
         <v>45139</v>
       </c>
@@ -9651,7 +9647,7 @@
       </c>
       <c r="E195" s="15"/>
     </row>
-    <row r="196" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="196" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A196" s="13">
         <v>45170</v>
       </c>
@@ -9663,7 +9659,7 @@
       </c>
       <c r="E196" s="15"/>
     </row>
-    <row r="197" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="197" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A197" s="13">
         <v>45200</v>
       </c>
@@ -9675,7 +9671,7 @@
       </c>
       <c r="E197" s="15"/>
     </row>
-    <row r="198" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="198" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A198" s="13">
         <v>45231</v>
       </c>
@@ -9687,7 +9683,7 @@
       </c>
       <c r="E198" s="15"/>
     </row>
-    <row r="199" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="199" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A199" s="13">
         <v>45261</v>
       </c>
@@ -9699,7 +9695,7 @@
       </c>
       <c r="E199" s="15"/>
     </row>
-    <row r="200" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="200" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A200" s="13">
         <v>45292</v>
       </c>
@@ -9711,7 +9707,7 @@
       </c>
       <c r="E200" s="15"/>
     </row>
-    <row r="201" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="201" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A201" s="13">
         <v>45323</v>
       </c>
@@ -9723,7 +9719,7 @@
       </c>
       <c r="E201" s="15"/>
     </row>
-    <row r="202" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="202" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A202" s="13">
         <v>45352</v>
       </c>
@@ -9735,7 +9731,7 @@
       </c>
       <c r="E202" s="15"/>
     </row>
-    <row r="203" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="203" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A203" s="13">
         <v>45383</v>
       </c>
@@ -9747,7 +9743,7 @@
       </c>
       <c r="E203" s="15"/>
     </row>
-    <row r="204" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="204" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A204" s="13">
         <v>45413</v>
       </c>
@@ -9759,7 +9755,7 @@
       </c>
       <c r="E204" s="15"/>
     </row>
-    <row r="205" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="205" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A205" s="13">
         <v>45444</v>
       </c>
@@ -9771,7 +9767,7 @@
       </c>
       <c r="E205" s="15"/>
     </row>
-    <row r="206" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="206" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A206" s="13">
         <v>45474</v>
       </c>
@@ -9783,7 +9779,7 @@
       </c>
       <c r="E206" s="15"/>
     </row>
-    <row r="207" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="207" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A207" s="13">
         <v>45505</v>
       </c>
@@ -9795,7 +9791,7 @@
       </c>
       <c r="E207" s="15"/>
     </row>
-    <row r="208" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="208" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A208" s="13">
         <v>45536</v>
       </c>
@@ -9807,7 +9803,7 @@
       </c>
       <c r="E208" s="15"/>
     </row>
-    <row r="209" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="209" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A209" s="13">
         <v>45566</v>
       </c>
@@ -9819,7 +9815,7 @@
       </c>
       <c r="E209" s="15"/>
     </row>
-    <row r="210" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="210" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A210" s="13">
         <v>45597</v>
       </c>
@@ -9831,7 +9827,7 @@
       </c>
       <c r="E210" s="15"/>
     </row>
-    <row r="211" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="211" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A211" s="13">
         <v>45627</v>
       </c>
@@ -9843,7 +9839,7 @@
       </c>
       <c r="E211" s="15"/>
     </row>
-    <row r="212" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="212" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A212" s="13">
         <v>45658</v>
       </c>
@@ -9855,7 +9851,7 @@
       </c>
       <c r="E212" s="15"/>
     </row>
-    <row r="213" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="213" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A213" s="13">
         <v>45689</v>
       </c>
@@ -9867,7 +9863,7 @@
       </c>
       <c r="E213" s="15"/>
     </row>
-    <row r="214" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="214" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A214" s="13">
         <v>45717</v>
       </c>
@@ -9878,7 +9874,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="215" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="215" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A215" s="13">
         <v>45748</v>
       </c>
@@ -9889,7 +9885,7 @@
         <v>-0.25</v>
       </c>
     </row>
-    <row r="216" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="216" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A216" s="13">
         <v>45778</v>
       </c>
@@ -9900,7 +9896,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="217" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="217" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A217" s="13">
         <v>45809</v>
       </c>
@@ -9921,22 +9917,22 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{508B4195-1E3B-44F9-B5F9-B093F5FD8600}">
   <dimension ref="A1:I285"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.44140625" defaultRowHeight="15.6" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="15.5703125" style="2" customWidth="1"/>
-    <col min="2" max="2" width="50.28515625" style="2" bestFit="1" customWidth="1"/>
-    <col min="3" max="16384" width="11.42578125" style="2"/>
+    <col min="1" max="1" width="15.5546875" style="2" customWidth="1"/>
+    <col min="2" max="2" width="50.33203125" style="2" bestFit="1" customWidth="1"/>
+    <col min="3" max="16384" width="11.44140625" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:9" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:9" ht="16.2" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A2" s="1"/>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A3" s="3" t="s">
         <v>6</v>
       </c>
@@ -9949,7 +9945,7 @@
       <c r="H3" s="4"/>
       <c r="I3" s="5"/>
     </row>
-    <row r="4" spans="1:9" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:9" ht="17.399999999999999" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A4" s="6" t="s">
         <v>7</v>
       </c>
@@ -9962,10 +9958,10 @@
       <c r="H4" s="7"/>
       <c r="I4" s="8"/>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A5" s="9"/>
     </row>
-    <row r="6" spans="1:9" ht="39.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:9" ht="39.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="10" t="s">
         <v>5</v>
       </c>
@@ -9973,7 +9969,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="7" spans="1:9" ht="17.25" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A7" s="12" t="s">
         <v>0</v>
       </c>
@@ -9981,7 +9977,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:9" s="13" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:9" s="13" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A8" s="13">
         <v>38047</v>
       </c>
@@ -9989,7 +9985,7 @@
         <v>0.12999999999999989</v>
       </c>
     </row>
-    <row r="9" spans="1:9" s="13" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:9" s="13" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A9" s="13">
         <v>38078</v>
       </c>
@@ -9997,7 +9993,7 @@
         <v>0.12000000000000011</v>
       </c>
     </row>
-    <row r="10" spans="1:9" s="13" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:9" s="13" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A10" s="13">
         <v>38108</v>
       </c>
@@ -10005,7 +10001,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:9" s="13" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:9" s="13" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A11" s="13">
         <v>38139</v>
       </c>
@@ -10013,7 +10009,7 @@
         <v>1.9999999999999574E-2</v>
       </c>
     </row>
-    <row r="12" spans="1:9" s="13" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:9" s="13" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A12" s="13">
         <v>38169</v>
       </c>
@@ -10021,7 +10017,7 @@
         <v>-1.9999999999999574E-2</v>
       </c>
     </row>
-    <row r="13" spans="1:9" s="13" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:9" s="13" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A13" s="13">
         <v>38200</v>
       </c>
@@ -10029,7 +10025,7 @@
         <v>-4.9999999999999822E-2</v>
       </c>
     </row>
-    <row r="14" spans="1:9" s="13" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:9" s="13" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A14" s="13">
         <v>38231</v>
       </c>
@@ -10037,7 +10033,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:9" s="13" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:9" s="13" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A15" s="13">
         <v>38261</v>
       </c>
@@ -10045,7 +10041,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:9" s="13" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:9" s="13" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A16" s="13">
         <v>38292</v>
       </c>
@@ -10053,7 +10049,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:2" s="13" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:2" s="13" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A17" s="13">
         <v>38322</v>
       </c>
@@ -10061,7 +10057,7 @@
         <v>-0.25</v>
       </c>
     </row>
-    <row r="18" spans="1:2" s="13" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:2" s="13" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A18" s="13">
         <v>38353</v>
       </c>
@@ -10069,7 +10065,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:2" s="13" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:2" s="13" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A19" s="13">
         <v>38384</v>
       </c>
@@ -10077,7 +10073,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:2" s="13" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:2" s="13" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A20" s="13">
         <v>38412</v>
       </c>
@@ -10085,7 +10081,7 @@
         <v>1.9999999999999574E-2</v>
       </c>
     </row>
-    <row r="21" spans="1:2" s="13" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:2" s="13" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A21" s="13">
         <v>38443</v>
       </c>
@@ -10093,7 +10089,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:2" s="13" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:2" s="13" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A22" s="13">
         <v>38473</v>
       </c>
@@ -10101,7 +10097,7 @@
         <v>9.9999999999997868E-3</v>
       </c>
     </row>
-    <row r="23" spans="1:2" s="13" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:2" s="13" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A23" s="13">
         <v>38504</v>
       </c>
@@ -10109,7 +10105,7 @@
         <v>1.9999999999999574E-2</v>
       </c>
     </row>
-    <row r="24" spans="1:2" s="13" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:2" s="13" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A24" s="13">
         <v>38534</v>
       </c>
@@ -10117,7 +10113,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:2" s="13" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:2" s="13" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A25" s="13">
         <v>38565</v>
       </c>
@@ -10125,7 +10121,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:2" s="13" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:2" s="13" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A26" s="13">
         <v>38596</v>
       </c>
@@ -10133,7 +10129,7 @@
         <v>-0.46999999999999975</v>
       </c>
     </row>
-    <row r="27" spans="1:2" s="13" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:2" s="13" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A27" s="13">
         <v>38626</v>
       </c>
@@ -10141,7 +10137,7 @@
         <v>8.0000000000000071E-2</v>
       </c>
     </row>
-    <row r="28" spans="1:2" s="13" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:2" s="13" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A28" s="13">
         <v>38657</v>
       </c>
@@ -10149,7 +10145,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:2" s="13" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:2" s="13" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A29" s="13">
         <v>38687</v>
       </c>
@@ -10157,7 +10153,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:2" s="13" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:2" s="13" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A30" s="13">
         <v>38718</v>
       </c>
@@ -10165,7 +10161,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:2" s="13" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:2" s="13" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A31" s="13">
         <v>38749</v>
       </c>
@@ -10173,7 +10169,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="32" spans="1:2" s="13" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:2" s="13" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A32" s="13">
         <v>38777</v>
       </c>
@@ -10181,7 +10177,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="33" spans="1:2" s="13" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:2" s="13" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A33" s="13">
         <v>38808</v>
       </c>
@@ -10189,7 +10185,7 @@
         <v>-1.9999999999999574E-2</v>
       </c>
     </row>
-    <row r="34" spans="1:2" s="13" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:2" s="13" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A34" s="13">
         <v>38838</v>
       </c>
@@ -10197,7 +10193,7 @@
         <v>-0.12999999999999989</v>
       </c>
     </row>
-    <row r="35" spans="1:2" s="13" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:2" s="13" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A35" s="13">
         <v>38869</v>
       </c>
@@ -10205,7 +10201,7 @@
         <v>4.0000000000000036E-2</v>
       </c>
     </row>
-    <row r="36" spans="1:2" s="13" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:2" s="13" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A36" s="13">
         <v>38899</v>
       </c>
@@ -10213,7 +10209,7 @@
         <v>-7.0000000000000284E-2</v>
       </c>
     </row>
-    <row r="37" spans="1:2" s="13" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:2" s="13" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A37" s="13">
         <v>38930</v>
       </c>
@@ -10221,7 +10217,7 @@
         <v>3.0000000000000249E-2</v>
       </c>
     </row>
-    <row r="38" spans="1:2" s="13" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:2" s="13" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A38" s="13">
         <v>38961</v>
       </c>
@@ -10229,7 +10225,7 @@
         <v>0.15000000000000036</v>
       </c>
     </row>
-    <row r="39" spans="1:2" s="13" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:2" s="13" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A39" s="13">
         <v>38991</v>
       </c>
@@ -10237,7 +10233,7 @@
         <v>8.0000000000000071E-2</v>
       </c>
     </row>
-    <row r="40" spans="1:2" s="13" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:2" s="13" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A40" s="13">
         <v>39022</v>
       </c>
@@ -10245,7 +10241,7 @@
         <v>-4.9999999999999822E-2</v>
       </c>
     </row>
-    <row r="41" spans="1:2" s="13" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:2" s="13" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A41" s="13">
         <v>39052</v>
       </c>
@@ -10253,7 +10249,7 @@
         <v>0.20000000000000018</v>
       </c>
     </row>
-    <row r="42" spans="1:2" s="13" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:2" s="13" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A42" s="13">
         <v>39083</v>
       </c>
@@ -10261,7 +10257,7 @@
         <v>0.12999999999999989</v>
       </c>
     </row>
-    <row r="43" spans="1:2" s="13" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:2" s="13" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A43" s="13">
         <v>39114</v>
       </c>
@@ -10269,7 +10265,7 @@
         <v>-1.9999999999999574E-2</v>
       </c>
     </row>
-    <row r="44" spans="1:2" s="13" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:2" s="13" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A44" s="13">
         <v>39142</v>
       </c>
@@ -10277,7 +10273,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" spans="1:2" s="13" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:2" s="13" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A45" s="13">
         <v>39173</v>
       </c>
@@ -10285,7 +10281,7 @@
         <v>-1.9999999999999574E-2</v>
       </c>
     </row>
-    <row r="46" spans="1:2" s="13" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:2" s="13" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A46" s="13">
         <v>39203</v>
       </c>
@@ -10293,7 +10289,7 @@
         <v>9.9999999999997868E-3</v>
       </c>
     </row>
-    <row r="47" spans="1:2" s="13" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:2" s="13" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A47" s="13">
         <v>39234</v>
       </c>
@@ -10301,7 +10297,7 @@
         <v>8.0000000000000071E-2</v>
       </c>
     </row>
-    <row r="48" spans="1:2" s="13" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:2" s="13" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A48" s="13">
         <v>39264</v>
       </c>
@@ -10309,7 +10305,7 @@
         <v>0.10999999999999943</v>
       </c>
     </row>
-    <row r="49" spans="1:4" s="13" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:4" s="13" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A49" s="13">
         <v>39295</v>
       </c>
@@ -10317,7 +10313,7 @@
         <v>-0.16000000000000014</v>
       </c>
     </row>
-    <row r="50" spans="1:4" s="13" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:4" s="13" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A50" s="13">
         <v>39326</v>
       </c>
@@ -10325,7 +10321,7 @@
         <v>-9.9999999999997868E-3</v>
       </c>
     </row>
-    <row r="51" spans="1:4" s="13" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:4" s="13" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A51" s="13">
         <v>39356</v>
       </c>
@@ -10333,7 +10329,7 @@
         <v>-9.9999999999997868E-3</v>
       </c>
     </row>
-    <row r="52" spans="1:4" s="13" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:4" s="13" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A52" s="13">
         <v>39387</v>
       </c>
@@ -10341,7 +10337,7 @@
         <v>0.24000000000000021</v>
       </c>
     </row>
-    <row r="53" spans="1:4" s="13" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:4" s="13" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A53" s="13">
         <v>39417</v>
       </c>
@@ -10349,7 +10345,7 @@
         <v>-9.9999999999997868E-3</v>
       </c>
     </row>
-    <row r="54" spans="1:4" s="13" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:4" s="13" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A54" s="13">
         <v>39448</v>
       </c>
@@ -10359,7 +10355,7 @@
       <c r="C54" s="19"/>
       <c r="D54" s="19"/>
     </row>
-    <row r="55" spans="1:4" s="13" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:4" s="13" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A55" s="13">
         <v>39479</v>
       </c>
@@ -10369,7 +10365,7 @@
       <c r="C55" s="19"/>
       <c r="D55" s="19"/>
     </row>
-    <row r="56" spans="1:4" s="13" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:4" s="13" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A56" s="13">
         <v>39508</v>
       </c>
@@ -10379,7 +10375,7 @@
       <c r="C56" s="19"/>
       <c r="D56" s="19"/>
     </row>
-    <row r="57" spans="1:4" s="13" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:4" s="13" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A57" s="13">
         <v>39539</v>
       </c>
@@ -10389,7 +10385,7 @@
       <c r="C57" s="19"/>
       <c r="D57" s="19"/>
     </row>
-    <row r="58" spans="1:4" s="13" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:4" s="13" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A58" s="13">
         <v>39569</v>
       </c>
@@ -10399,7 +10395,7 @@
       <c r="C58" s="19"/>
       <c r="D58" s="19"/>
     </row>
-    <row r="59" spans="1:4" s="13" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:4" s="13" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A59" s="13">
         <v>39600</v>
       </c>
@@ -10409,7 +10405,7 @@
       <c r="C59" s="19"/>
       <c r="D59" s="19"/>
     </row>
-    <row r="60" spans="1:4" s="13" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:4" s="13" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A60" s="13">
         <v>39630</v>
       </c>
@@ -10419,7 +10415,7 @@
       <c r="C60" s="19"/>
       <c r="D60" s="19"/>
     </row>
-    <row r="61" spans="1:4" s="13" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:4" s="13" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A61" s="13">
         <v>39661</v>
       </c>
@@ -10429,7 +10425,7 @@
       <c r="C61" s="19"/>
       <c r="D61" s="19"/>
     </row>
-    <row r="62" spans="1:4" s="13" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:4" s="13" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A62" s="13">
         <v>39692</v>
       </c>
@@ -10439,7 +10435,7 @@
       <c r="C62" s="19"/>
       <c r="D62" s="19"/>
     </row>
-    <row r="63" spans="1:4" s="13" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:4" s="13" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A63" s="13">
         <v>39722</v>
       </c>
@@ -10449,7 +10445,7 @@
       <c r="C63" s="19"/>
       <c r="D63" s="19"/>
     </row>
-    <row r="64" spans="1:4" s="13" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:4" s="13" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A64" s="13">
         <v>39753</v>
       </c>
@@ -10459,7 +10455,7 @@
       <c r="C64" s="19"/>
       <c r="D64" s="19"/>
     </row>
-    <row r="65" spans="1:4" s="13" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:4" s="13" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A65" s="13">
         <v>39783</v>
       </c>
@@ -10469,7 +10465,7 @@
       <c r="C65" s="19"/>
       <c r="D65" s="19"/>
     </row>
-    <row r="66" spans="1:4" s="13" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:4" s="13" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A66" s="13">
         <v>39814</v>
       </c>
@@ -10479,7 +10475,7 @@
       <c r="C66" s="19"/>
       <c r="D66" s="19"/>
     </row>
-    <row r="67" spans="1:4" s="13" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:4" s="13" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A67" s="13">
         <v>39845</v>
       </c>
@@ -10489,7 +10485,7 @@
       <c r="C67" s="19"/>
       <c r="D67" s="19"/>
     </row>
-    <row r="68" spans="1:4" s="13" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:4" s="13" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A68" s="13">
         <v>39873</v>
       </c>
@@ -10499,7 +10495,7 @@
       <c r="C68" s="19"/>
       <c r="D68" s="19"/>
     </row>
-    <row r="69" spans="1:4" s="13" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:4" s="13" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A69" s="13">
         <v>39904</v>
       </c>
@@ -10509,7 +10505,7 @@
       <c r="C69" s="19"/>
       <c r="D69" s="19"/>
     </row>
-    <row r="70" spans="1:4" s="13" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:4" s="13" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A70" s="13">
         <v>39934</v>
       </c>
@@ -10519,7 +10515,7 @@
       <c r="C70" s="19"/>
       <c r="D70" s="19"/>
     </row>
-    <row r="71" spans="1:4" s="13" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:4" s="13" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A71" s="13">
         <v>39965</v>
       </c>
@@ -10529,7 +10525,7 @@
       <c r="C71" s="19"/>
       <c r="D71" s="19"/>
     </row>
-    <row r="72" spans="1:4" s="13" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:4" s="13" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A72" s="13">
         <v>39995</v>
       </c>
@@ -10539,7 +10535,7 @@
       <c r="C72" s="19"/>
       <c r="D72" s="19"/>
     </row>
-    <row r="73" spans="1:4" s="13" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:4" s="13" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A73" s="13">
         <v>40026</v>
       </c>
@@ -10549,7 +10545,7 @@
       <c r="C73" s="19"/>
       <c r="D73" s="19"/>
     </row>
-    <row r="74" spans="1:4" s="13" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:4" s="13" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A74" s="13">
         <v>40057</v>
       </c>
@@ -10559,7 +10555,7 @@
       <c r="C74" s="19"/>
       <c r="D74" s="19"/>
     </row>
-    <row r="75" spans="1:4" s="13" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:4" s="13" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A75" s="13">
         <v>40087</v>
       </c>
@@ -10569,7 +10565,7 @@
       <c r="C75" s="19"/>
       <c r="D75" s="19"/>
     </row>
-    <row r="76" spans="1:4" s="13" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:4" s="13" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A76" s="13">
         <v>40118</v>
       </c>
@@ -10579,7 +10575,7 @@
       <c r="C76" s="19"/>
       <c r="D76" s="19"/>
     </row>
-    <row r="77" spans="1:4" s="13" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:4" s="13" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A77" s="13">
         <v>40148</v>
       </c>
@@ -10589,7 +10585,7 @@
       <c r="C77" s="19"/>
       <c r="D77" s="19"/>
     </row>
-    <row r="78" spans="1:4" ht="17.25" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A78" s="13">
         <v>40179</v>
       </c>
@@ -10599,7 +10595,7 @@
       <c r="C78" s="21"/>
       <c r="D78" s="19"/>
     </row>
-    <row r="79" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A79" s="13">
         <v>40210</v>
       </c>
@@ -10609,7 +10605,7 @@
       <c r="C79" s="21"/>
       <c r="D79" s="19"/>
     </row>
-    <row r="80" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A80" s="13">
         <v>40238</v>
       </c>
@@ -10619,7 +10615,7 @@
       <c r="C80" s="21"/>
       <c r="D80" s="19"/>
     </row>
-    <row r="81" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A81" s="13">
         <v>40269</v>
       </c>
@@ -10629,7 +10625,7 @@
       <c r="C81" s="21"/>
       <c r="D81" s="19"/>
     </row>
-    <row r="82" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A82" s="13">
         <v>40299</v>
       </c>
@@ -10639,7 +10635,7 @@
       <c r="C82" s="21"/>
       <c r="D82" s="19"/>
     </row>
-    <row r="83" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A83" s="13">
         <v>40330</v>
       </c>
@@ -10649,7 +10645,7 @@
       <c r="C83" s="21"/>
       <c r="D83" s="19"/>
     </row>
-    <row r="84" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A84" s="13">
         <v>40360</v>
       </c>
@@ -10659,7 +10655,7 @@
       <c r="C84" s="21"/>
       <c r="D84" s="19"/>
     </row>
-    <row r="85" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A85" s="13">
         <v>40391</v>
       </c>
@@ -10669,7 +10665,7 @@
       <c r="C85" s="21"/>
       <c r="D85" s="19"/>
     </row>
-    <row r="86" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A86" s="13">
         <v>40422</v>
       </c>
@@ -10679,7 +10675,7 @@
       <c r="C86" s="21"/>
       <c r="D86" s="19"/>
     </row>
-    <row r="87" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A87" s="13">
         <v>40452</v>
       </c>
@@ -10689,7 +10685,7 @@
       <c r="C87" s="21"/>
       <c r="D87" s="19"/>
     </row>
-    <row r="88" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A88" s="13">
         <v>40483</v>
       </c>
@@ -10699,7 +10695,7 @@
       <c r="C88" s="21"/>
       <c r="D88" s="19"/>
     </row>
-    <row r="89" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A89" s="13">
         <v>40513</v>
       </c>
@@ -10709,7 +10705,7 @@
       <c r="C89" s="21"/>
       <c r="D89" s="19"/>
     </row>
-    <row r="90" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A90" s="13">
         <v>40544</v>
       </c>
@@ -10719,7 +10715,7 @@
       <c r="C90" s="21"/>
       <c r="D90" s="19"/>
     </row>
-    <row r="91" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A91" s="13">
         <v>40575</v>
       </c>
@@ -10729,7 +10725,7 @@
       <c r="C91" s="21"/>
       <c r="D91" s="19"/>
     </row>
-    <row r="92" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A92" s="13">
         <v>40603</v>
       </c>
@@ -10739,7 +10735,7 @@
       <c r="C92" s="21"/>
       <c r="D92" s="19"/>
     </row>
-    <row r="93" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A93" s="13">
         <v>40634</v>
       </c>
@@ -10749,7 +10745,7 @@
       <c r="C93" s="21"/>
       <c r="D93" s="19"/>
     </row>
-    <row r="94" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A94" s="13">
         <v>40664</v>
       </c>
@@ -10759,7 +10755,7 @@
       <c r="C94" s="21"/>
       <c r="D94" s="19"/>
     </row>
-    <row r="95" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A95" s="13">
         <v>40695</v>
       </c>
@@ -10769,7 +10765,7 @@
       <c r="C95" s="21"/>
       <c r="D95" s="19"/>
     </row>
-    <row r="96" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A96" s="13">
         <v>40725</v>
       </c>
@@ -10779,7 +10775,7 @@
       <c r="C96" s="21"/>
       <c r="D96" s="19"/>
     </row>
-    <row r="97" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A97" s="13">
         <v>40756</v>
       </c>
@@ -10789,7 +10785,7 @@
       <c r="C97" s="21"/>
       <c r="D97" s="19"/>
     </row>
-    <row r="98" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A98" s="13">
         <v>40787</v>
       </c>
@@ -10799,7 +10795,7 @@
       <c r="C98" s="21"/>
       <c r="D98" s="19"/>
     </row>
-    <row r="99" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A99" s="13">
         <v>40817</v>
       </c>
@@ -10809,7 +10805,7 @@
       <c r="C99" s="21"/>
       <c r="D99" s="19"/>
     </row>
-    <row r="100" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A100" s="13">
         <v>40848</v>
       </c>
@@ -10819,7 +10815,7 @@
       <c r="C100" s="21"/>
       <c r="D100" s="19"/>
     </row>
-    <row r="101" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A101" s="13">
         <v>40878</v>
       </c>
@@ -10829,7 +10825,7 @@
       <c r="C101" s="21"/>
       <c r="D101" s="19"/>
     </row>
-    <row r="102" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A102" s="13">
         <v>40909</v>
       </c>
@@ -10839,7 +10835,7 @@
       <c r="C102" s="21"/>
       <c r="D102" s="19"/>
     </row>
-    <row r="103" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A103" s="13">
         <v>40940</v>
       </c>
@@ -10849,7 +10845,7 @@
       <c r="C103" s="21"/>
       <c r="D103" s="19"/>
     </row>
-    <row r="104" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A104" s="13">
         <v>40969</v>
       </c>
@@ -10859,7 +10855,7 @@
       <c r="C104" s="21"/>
       <c r="D104" s="19"/>
     </row>
-    <row r="105" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A105" s="13">
         <v>41000</v>
       </c>
@@ -10869,7 +10865,7 @@
       <c r="C105" s="21"/>
       <c r="D105" s="19"/>
     </row>
-    <row r="106" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A106" s="13">
         <v>41030</v>
       </c>
@@ -10879,7 +10875,7 @@
       <c r="C106" s="21"/>
       <c r="D106" s="19"/>
     </row>
-    <row r="107" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A107" s="13">
         <v>41061</v>
       </c>
@@ -10889,7 +10885,7 @@
       <c r="C107" s="21"/>
       <c r="D107" s="19"/>
     </row>
-    <row r="108" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A108" s="13">
         <v>41091</v>
       </c>
@@ -10899,7 +10895,7 @@
       <c r="C108" s="21"/>
       <c r="D108" s="19"/>
     </row>
-    <row r="109" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A109" s="13">
         <v>41122</v>
       </c>
@@ -10909,7 +10905,7 @@
       <c r="C109" s="21"/>
       <c r="D109" s="19"/>
     </row>
-    <row r="110" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A110" s="13">
         <v>41153</v>
       </c>
@@ -10919,7 +10915,7 @@
       <c r="C110" s="21"/>
       <c r="D110" s="19"/>
     </row>
-    <row r="111" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A111" s="13">
         <v>41183</v>
       </c>
@@ -10929,7 +10925,7 @@
       <c r="C111" s="21"/>
       <c r="D111" s="19"/>
     </row>
-    <row r="112" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A112" s="13">
         <v>41214</v>
       </c>
@@ -10939,7 +10935,7 @@
       <c r="C112" s="21"/>
       <c r="D112" s="19"/>
     </row>
-    <row r="113" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="113" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A113" s="13">
         <v>41244</v>
       </c>
@@ -10949,7 +10945,7 @@
       <c r="C113" s="21"/>
       <c r="D113" s="19"/>
     </row>
-    <row r="114" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="114" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A114" s="13">
         <v>41275</v>
       </c>
@@ -10959,7 +10955,7 @@
       <c r="C114" s="21"/>
       <c r="D114" s="19"/>
     </row>
-    <row r="115" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A115" s="13">
         <v>41306</v>
       </c>
@@ -10969,7 +10965,7 @@
       <c r="C115" s="21"/>
       <c r="D115" s="19"/>
     </row>
-    <row r="116" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="116" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A116" s="13">
         <v>41334</v>
       </c>
@@ -10979,7 +10975,7 @@
       <c r="C116" s="21"/>
       <c r="D116" s="19"/>
     </row>
-    <row r="117" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="117" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A117" s="13">
         <v>41365</v>
       </c>
@@ -10989,7 +10985,7 @@
       <c r="C117" s="21"/>
       <c r="D117" s="19"/>
     </row>
-    <row r="118" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="118" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A118" s="13">
         <v>41395</v>
       </c>
@@ -10999,7 +10995,7 @@
       <c r="C118" s="21"/>
       <c r="D118" s="19"/>
     </row>
-    <row r="119" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="119" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A119" s="13">
         <v>41426</v>
       </c>
@@ -11009,7 +11005,7 @@
       <c r="C119" s="21"/>
       <c r="D119" s="19"/>
     </row>
-    <row r="120" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="120" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A120" s="13">
         <v>41456</v>
       </c>
@@ -11019,7 +11015,7 @@
       <c r="C120" s="21"/>
       <c r="D120" s="19"/>
     </row>
-    <row r="121" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="121" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A121" s="13">
         <v>41487</v>
       </c>
@@ -11029,7 +11025,7 @@
       <c r="C121" s="21"/>
       <c r="D121" s="19"/>
     </row>
-    <row r="122" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="122" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A122" s="13">
         <v>41518</v>
       </c>
@@ -11039,7 +11035,7 @@
       <c r="C122" s="21"/>
       <c r="D122" s="19"/>
     </row>
-    <row r="123" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="123" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A123" s="13">
         <v>41548</v>
       </c>
@@ -11049,7 +11045,7 @@
       <c r="C123" s="21"/>
       <c r="D123" s="19"/>
     </row>
-    <row r="124" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="124" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A124" s="13">
         <v>41579</v>
       </c>
@@ -11059,7 +11055,7 @@
       <c r="C124" s="21"/>
       <c r="D124" s="19"/>
     </row>
-    <row r="125" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="125" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A125" s="13">
         <v>41609</v>
       </c>
@@ -11069,7 +11065,7 @@
       <c r="C125" s="21"/>
       <c r="D125" s="19"/>
     </row>
-    <row r="126" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="126" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A126" s="13">
         <v>41640</v>
       </c>
@@ -11079,7 +11075,7 @@
       <c r="C126" s="21"/>
       <c r="D126" s="19"/>
     </row>
-    <row r="127" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="127" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A127" s="13">
         <v>41671</v>
       </c>
@@ -11089,7 +11085,7 @@
       <c r="C127" s="21"/>
       <c r="D127" s="19"/>
     </row>
-    <row r="128" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="128" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A128" s="13">
         <v>41699</v>
       </c>
@@ -11099,7 +11095,7 @@
       <c r="C128" s="21"/>
       <c r="D128" s="19"/>
     </row>
-    <row r="129" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="129" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A129" s="13">
         <v>41730</v>
       </c>
@@ -11109,7 +11105,7 @@
       <c r="C129" s="21"/>
       <c r="D129" s="19"/>
     </row>
-    <row r="130" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="130" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A130" s="13">
         <v>41760</v>
       </c>
@@ -11119,7 +11115,7 @@
       <c r="C130" s="21"/>
       <c r="D130" s="19"/>
     </row>
-    <row r="131" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="131" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A131" s="13">
         <v>41791</v>
       </c>
@@ -11129,7 +11125,7 @@
       <c r="C131" s="21"/>
       <c r="D131" s="19"/>
     </row>
-    <row r="132" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="132" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A132" s="13">
         <v>41821</v>
       </c>
@@ -11139,7 +11135,7 @@
       <c r="C132" s="21"/>
       <c r="D132" s="19"/>
     </row>
-    <row r="133" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="133" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A133" s="13">
         <v>41852</v>
       </c>
@@ -11149,7 +11145,7 @@
       <c r="C133" s="21"/>
       <c r="D133" s="19"/>
     </row>
-    <row r="134" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="134" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A134" s="13">
         <v>41883</v>
       </c>
@@ -11159,7 +11155,7 @@
       <c r="C134" s="21"/>
       <c r="D134" s="19"/>
     </row>
-    <row r="135" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="135" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A135" s="13">
         <v>41913</v>
       </c>
@@ -11169,7 +11165,7 @@
       <c r="C135" s="21"/>
       <c r="D135" s="19"/>
     </row>
-    <row r="136" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="136" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A136" s="13">
         <v>41944</v>
       </c>
@@ -11179,7 +11175,7 @@
       <c r="C136" s="21"/>
       <c r="D136" s="19"/>
     </row>
-    <row r="137" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="137" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A137" s="13">
         <v>41974</v>
       </c>
@@ -11189,7 +11185,7 @@
       <c r="C137" s="21"/>
       <c r="D137" s="19"/>
     </row>
-    <row r="138" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="138" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A138" s="13">
         <v>42005</v>
       </c>
@@ -11199,7 +11195,7 @@
       <c r="C138" s="21"/>
       <c r="D138" s="19"/>
     </row>
-    <row r="139" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="139" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A139" s="13">
         <v>42036</v>
       </c>
@@ -11209,7 +11205,7 @@
       <c r="C139" s="21"/>
       <c r="D139" s="19"/>
     </row>
-    <row r="140" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="140" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A140" s="13">
         <v>42064</v>
       </c>
@@ -11219,7 +11215,7 @@
       <c r="C140" s="21"/>
       <c r="D140" s="19"/>
     </row>
-    <row r="141" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="141" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A141" s="13">
         <v>42095</v>
       </c>
@@ -11229,7 +11225,7 @@
       <c r="C141" s="21"/>
       <c r="D141" s="19"/>
     </row>
-    <row r="142" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="142" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A142" s="13">
         <v>42125</v>
       </c>
@@ -11239,7 +11235,7 @@
       <c r="C142" s="21"/>
       <c r="D142" s="19"/>
     </row>
-    <row r="143" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="143" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A143" s="13">
         <v>42156</v>
       </c>
@@ -11249,7 +11245,7 @@
       <c r="C143" s="21"/>
       <c r="D143" s="19"/>
     </row>
-    <row r="144" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="144" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A144" s="13">
         <v>42186</v>
       </c>
@@ -11259,7 +11255,7 @@
       <c r="C144" s="21"/>
       <c r="D144" s="19"/>
     </row>
-    <row r="145" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="145" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A145" s="13">
         <v>42217</v>
       </c>
@@ -11269,7 +11265,7 @@
       <c r="C145" s="21"/>
       <c r="D145" s="19"/>
     </row>
-    <row r="146" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="146" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A146" s="13">
         <v>42248</v>
       </c>
@@ -11279,7 +11275,7 @@
       <c r="C146" s="21"/>
       <c r="D146" s="19"/>
     </row>
-    <row r="147" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="147" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A147" s="13">
         <v>42278</v>
       </c>
@@ -11289,7 +11285,7 @@
       <c r="C147" s="21"/>
       <c r="D147" s="19"/>
     </row>
-    <row r="148" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="148" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A148" s="13">
         <v>42309</v>
       </c>
@@ -11299,7 +11295,7 @@
       <c r="C148" s="21"/>
       <c r="D148" s="19"/>
     </row>
-    <row r="149" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="149" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A149" s="13">
         <v>42339</v>
       </c>
@@ -11309,7 +11305,7 @@
       <c r="C149" s="21"/>
       <c r="D149" s="19"/>
     </row>
-    <row r="150" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="150" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A150" s="13">
         <v>42370</v>
       </c>
@@ -11319,7 +11315,7 @@
       <c r="C150" s="21"/>
       <c r="D150" s="19"/>
     </row>
-    <row r="151" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="151" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A151" s="13">
         <v>42401</v>
       </c>
@@ -11329,7 +11325,7 @@
       <c r="C151" s="21"/>
       <c r="D151" s="19"/>
     </row>
-    <row r="152" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="152" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A152" s="13">
         <v>42430</v>
       </c>
@@ -11339,7 +11335,7 @@
       <c r="C152" s="21"/>
       <c r="D152" s="19"/>
     </row>
-    <row r="153" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="153" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A153" s="13">
         <v>42461</v>
       </c>
@@ -11349,7 +11345,7 @@
       <c r="C153" s="21"/>
       <c r="D153" s="19"/>
     </row>
-    <row r="154" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="154" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A154" s="13">
         <v>42491</v>
       </c>
@@ -11359,7 +11355,7 @@
       <c r="C154" s="21"/>
       <c r="D154" s="19"/>
     </row>
-    <row r="155" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="155" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A155" s="13">
         <v>42522</v>
       </c>
@@ -11369,7 +11365,7 @@
       <c r="C155" s="21"/>
       <c r="D155" s="19"/>
     </row>
-    <row r="156" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="156" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A156" s="13">
         <v>42552</v>
       </c>
@@ -11379,7 +11375,7 @@
       <c r="C156" s="21"/>
       <c r="D156" s="19"/>
     </row>
-    <row r="157" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="157" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A157" s="13">
         <v>42583</v>
       </c>
@@ -11389,7 +11385,7 @@
       <c r="C157" s="21"/>
       <c r="D157" s="19"/>
     </row>
-    <row r="158" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="158" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A158" s="13">
         <v>42614</v>
       </c>
@@ -11399,7 +11395,7 @@
       <c r="C158" s="21"/>
       <c r="D158" s="19"/>
     </row>
-    <row r="159" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="159" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A159" s="13">
         <v>42644</v>
       </c>
@@ -11409,7 +11405,7 @@
       <c r="C159" s="21"/>
       <c r="D159" s="19"/>
     </row>
-    <row r="160" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="160" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A160" s="13">
         <v>42675</v>
       </c>
@@ -11419,7 +11415,7 @@
       <c r="C160" s="21"/>
       <c r="D160" s="19"/>
     </row>
-    <row r="161" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="161" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A161" s="13">
         <v>42705</v>
       </c>
@@ -11429,7 +11425,7 @@
       <c r="C161" s="21"/>
       <c r="D161" s="19"/>
     </row>
-    <row r="162" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="162" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A162" s="13">
         <v>42736</v>
       </c>
@@ -11439,7 +11435,7 @@
       <c r="C162" s="21"/>
       <c r="D162" s="19"/>
     </row>
-    <row r="163" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="163" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A163" s="13">
         <v>42767</v>
       </c>
@@ -11449,7 +11445,7 @@
       <c r="C163" s="21"/>
       <c r="D163" s="19"/>
     </row>
-    <row r="164" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="164" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A164" s="13">
         <v>42795</v>
       </c>
@@ -11459,7 +11455,7 @@
       <c r="C164" s="21"/>
       <c r="D164" s="19"/>
     </row>
-    <row r="165" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="165" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A165" s="13">
         <v>42826</v>
       </c>
@@ -11469,7 +11465,7 @@
       <c r="C165" s="21"/>
       <c r="D165" s="19"/>
     </row>
-    <row r="166" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="166" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A166" s="13">
         <v>42856</v>
       </c>
@@ -11479,7 +11475,7 @@
       <c r="C166" s="21"/>
       <c r="D166" s="19"/>
     </row>
-    <row r="167" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="167" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A167" s="13">
         <v>42887</v>
       </c>
@@ -11489,7 +11485,7 @@
       <c r="C167" s="21"/>
       <c r="D167" s="19"/>
     </row>
-    <row r="168" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="168" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A168" s="13">
         <v>42917</v>
       </c>
@@ -11499,7 +11495,7 @@
       <c r="C168" s="21"/>
       <c r="D168" s="19"/>
     </row>
-    <row r="169" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="169" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A169" s="13">
         <v>42948</v>
       </c>
@@ -11509,7 +11505,7 @@
       <c r="C169" s="21"/>
       <c r="D169" s="19"/>
     </row>
-    <row r="170" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="170" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A170" s="13">
         <v>42979</v>
       </c>
@@ -11519,7 +11515,7 @@
       <c r="C170" s="21"/>
       <c r="D170" s="19"/>
     </row>
-    <row r="171" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="171" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A171" s="13">
         <v>43009</v>
       </c>
@@ -11529,7 +11525,7 @@
       <c r="C171" s="21"/>
       <c r="D171" s="19"/>
     </row>
-    <row r="172" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="172" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A172" s="13">
         <v>43040</v>
       </c>
@@ -11539,7 +11535,7 @@
       <c r="C172" s="21"/>
       <c r="D172" s="19"/>
     </row>
-    <row r="173" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="173" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A173" s="13">
         <v>43070</v>
       </c>
@@ -11549,7 +11545,7 @@
       <c r="C173" s="21"/>
       <c r="D173" s="19"/>
     </row>
-    <row r="174" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="174" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A174" s="13">
         <v>43101</v>
       </c>
@@ -11559,7 +11555,7 @@
       <c r="C174" s="21"/>
       <c r="D174" s="19"/>
     </row>
-    <row r="175" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="175" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A175" s="13">
         <v>43132</v>
       </c>
@@ -11569,7 +11565,7 @@
       <c r="C175" s="21"/>
       <c r="D175" s="19"/>
     </row>
-    <row r="176" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="176" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A176" s="13">
         <v>43160</v>
       </c>
@@ -11579,7 +11575,7 @@
       <c r="C176" s="21"/>
       <c r="D176" s="19"/>
     </row>
-    <row r="177" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="177" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A177" s="13">
         <v>43191</v>
       </c>
@@ -11589,7 +11585,7 @@
       <c r="C177" s="21"/>
       <c r="D177" s="19"/>
     </row>
-    <row r="178" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="178" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A178" s="13">
         <v>43221</v>
       </c>
@@ -11599,7 +11595,7 @@
       <c r="C178" s="21"/>
       <c r="D178" s="19"/>
     </row>
-    <row r="179" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="179" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A179" s="13">
         <v>43252</v>
       </c>
@@ -11609,7 +11605,7 @@
       <c r="C179" s="21"/>
       <c r="D179" s="19"/>
     </row>
-    <row r="180" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="180" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A180" s="13">
         <v>43282</v>
       </c>
@@ -11619,7 +11615,7 @@
       <c r="C180" s="21"/>
       <c r="D180" s="19"/>
     </row>
-    <row r="181" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="181" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A181" s="13">
         <v>43313</v>
       </c>
@@ -11629,7 +11625,7 @@
       <c r="C181" s="21"/>
       <c r="D181" s="19"/>
     </row>
-    <row r="182" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="182" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A182" s="13">
         <v>43344</v>
       </c>
@@ -11639,7 +11635,7 @@
       <c r="C182" s="21"/>
       <c r="D182" s="19"/>
     </row>
-    <row r="183" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="183" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A183" s="13">
         <v>43374</v>
       </c>
@@ -11649,7 +11645,7 @@
       <c r="C183" s="21"/>
       <c r="D183" s="19"/>
     </row>
-    <row r="184" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="184" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A184" s="13">
         <v>43405</v>
       </c>
@@ -11659,7 +11655,7 @@
       <c r="C184" s="21"/>
       <c r="D184" s="19"/>
     </row>
-    <row r="185" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="185" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A185" s="13">
         <v>43435</v>
       </c>
@@ -11669,7 +11665,7 @@
       <c r="C185" s="21"/>
       <c r="D185" s="19"/>
     </row>
-    <row r="186" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="186" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A186" s="13">
         <v>43466</v>
       </c>
@@ -11679,7 +11675,7 @@
       <c r="C186" s="21"/>
       <c r="D186" s="19"/>
     </row>
-    <row r="187" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="187" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A187" s="13">
         <v>43497</v>
       </c>
@@ -11689,7 +11685,7 @@
       <c r="C187" s="21"/>
       <c r="D187" s="19"/>
     </row>
-    <row r="188" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="188" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A188" s="13">
         <v>43525</v>
       </c>
@@ -11699,7 +11695,7 @@
       <c r="C188" s="21"/>
       <c r="D188" s="19"/>
     </row>
-    <row r="189" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="189" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A189" s="13">
         <v>43556</v>
       </c>
@@ -11709,7 +11705,7 @@
       <c r="C189" s="21"/>
       <c r="D189" s="19"/>
     </row>
-    <row r="190" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="190" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A190" s="13">
         <v>43586</v>
       </c>
@@ -11719,7 +11715,7 @@
       <c r="C190" s="21"/>
       <c r="D190" s="19"/>
     </row>
-    <row r="191" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="191" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A191" s="13">
         <v>43617</v>
       </c>
@@ -11729,7 +11725,7 @@
       <c r="C191" s="21"/>
       <c r="D191" s="19"/>
     </row>
-    <row r="192" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="192" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A192" s="13">
         <v>43647</v>
       </c>
@@ -11739,7 +11735,7 @@
       <c r="C192" s="21"/>
       <c r="D192" s="19"/>
     </row>
-    <row r="193" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="193" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A193" s="13">
         <v>43678</v>
       </c>
@@ -11749,7 +11745,7 @@
       <c r="C193" s="21"/>
       <c r="D193" s="19"/>
     </row>
-    <row r="194" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="194" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A194" s="13">
         <v>43709</v>
       </c>
@@ -11759,7 +11755,7 @@
       <c r="C194" s="21"/>
       <c r="D194" s="19"/>
     </row>
-    <row r="195" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="195" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A195" s="13">
         <v>43739</v>
       </c>
@@ -11769,7 +11765,7 @@
       <c r="C195" s="21"/>
       <c r="D195" s="19"/>
     </row>
-    <row r="196" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="196" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A196" s="13">
         <v>43770</v>
       </c>
@@ -11779,7 +11775,7 @@
       <c r="C196" s="21"/>
       <c r="D196" s="19"/>
     </row>
-    <row r="197" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="197" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A197" s="13">
         <v>43800</v>
       </c>
@@ -11789,7 +11785,7 @@
       <c r="C197" s="21"/>
       <c r="D197" s="19"/>
     </row>
-    <row r="198" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="198" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A198" s="13">
         <v>43831</v>
       </c>
@@ -11799,7 +11795,7 @@
       <c r="C198" s="21"/>
       <c r="D198" s="19"/>
     </row>
-    <row r="199" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="199" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A199" s="13">
         <v>43862</v>
       </c>
@@ -11809,7 +11805,7 @@
       <c r="C199" s="21"/>
       <c r="D199" s="19"/>
     </row>
-    <row r="200" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="200" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A200" s="13">
         <v>43891</v>
       </c>
@@ -11819,7 +11815,7 @@
       <c r="C200" s="21"/>
       <c r="D200" s="19"/>
     </row>
-    <row r="201" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="201" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A201" s="13">
         <v>43922</v>
       </c>
@@ -11829,7 +11825,7 @@
       <c r="C201" s="21"/>
       <c r="D201" s="19"/>
     </row>
-    <row r="202" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="202" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A202" s="13">
         <v>43952</v>
       </c>
@@ -11839,7 +11835,7 @@
       <c r="C202" s="21"/>
       <c r="D202" s="19"/>
     </row>
-    <row r="203" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="203" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A203" s="13">
         <v>43983</v>
       </c>
@@ -11849,7 +11845,7 @@
       <c r="C203" s="21"/>
       <c r="D203" s="19"/>
     </row>
-    <row r="204" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="204" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A204" s="13">
         <v>44013</v>
       </c>
@@ -11859,7 +11855,7 @@
       <c r="C204" s="21"/>
       <c r="D204" s="19"/>
     </row>
-    <row r="205" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="205" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A205" s="13">
         <v>44044</v>
       </c>
@@ -11869,7 +11865,7 @@
       <c r="C205" s="21"/>
       <c r="D205" s="19"/>
     </row>
-    <row r="206" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="206" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A206" s="13">
         <v>44075</v>
       </c>
@@ -11879,7 +11875,7 @@
       <c r="C206" s="21"/>
       <c r="D206" s="19"/>
     </row>
-    <row r="207" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="207" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A207" s="13">
         <v>44105</v>
       </c>
@@ -11889,7 +11885,7 @@
       <c r="C207" s="21"/>
       <c r="D207" s="19"/>
     </row>
-    <row r="208" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="208" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A208" s="13">
         <v>44136</v>
       </c>
@@ -11899,7 +11895,7 @@
       <c r="C208" s="21"/>
       <c r="D208" s="19"/>
     </row>
-    <row r="209" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="209" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A209" s="13">
         <v>44166</v>
       </c>
@@ -11909,7 +11905,7 @@
       <c r="C209" s="21"/>
       <c r="D209" s="19"/>
     </row>
-    <row r="210" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="210" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A210" s="13">
         <v>44197</v>
       </c>
@@ -11919,7 +11915,7 @@
       <c r="C210" s="21"/>
       <c r="D210" s="19"/>
     </row>
-    <row r="211" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="211" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A211" s="13">
         <v>44228</v>
       </c>
@@ -11929,7 +11925,7 @@
       <c r="C211" s="21"/>
       <c r="D211" s="19"/>
     </row>
-    <row r="212" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="212" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A212" s="13">
         <v>44256</v>
       </c>
@@ -11939,7 +11935,7 @@
       <c r="C212" s="21"/>
       <c r="D212" s="19"/>
     </row>
-    <row r="213" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="213" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A213" s="13">
         <v>44287</v>
       </c>
@@ -11949,7 +11945,7 @@
       <c r="C213" s="21"/>
       <c r="D213" s="19"/>
     </row>
-    <row r="214" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="214" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A214" s="13">
         <v>44317</v>
       </c>
@@ -11959,7 +11955,7 @@
       <c r="C214" s="21"/>
       <c r="D214" s="19"/>
     </row>
-    <row r="215" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="215" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A215" s="13">
         <v>44348</v>
       </c>
@@ -11969,7 +11965,7 @@
       <c r="C215" s="21"/>
       <c r="D215" s="19"/>
     </row>
-    <row r="216" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="216" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A216" s="13">
         <v>44378</v>
       </c>
@@ -11979,7 +11975,7 @@
       <c r="C216" s="21"/>
       <c r="D216" s="19"/>
     </row>
-    <row r="217" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="217" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A217" s="13">
         <v>44409</v>
       </c>
@@ -11989,7 +11985,7 @@
       <c r="C217" s="21"/>
       <c r="D217" s="19"/>
     </row>
-    <row r="218" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="218" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A218" s="13">
         <v>44440</v>
       </c>
@@ -11999,7 +11995,7 @@
       <c r="C218" s="21"/>
       <c r="D218" s="19"/>
     </row>
-    <row r="219" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="219" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A219" s="13">
         <v>44470</v>
       </c>
@@ -12009,7 +12005,7 @@
       <c r="C219" s="21"/>
       <c r="D219" s="19"/>
     </row>
-    <row r="220" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="220" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A220" s="13">
         <v>44501</v>
       </c>
@@ -12019,7 +12015,7 @@
       <c r="C220" s="21"/>
       <c r="D220" s="19"/>
     </row>
-    <row r="221" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="221" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A221" s="13">
         <v>44531</v>
       </c>
@@ -12029,7 +12025,7 @@
       <c r="C221" s="21"/>
       <c r="D221" s="19"/>
     </row>
-    <row r="222" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="222" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A222" s="13">
         <v>44562</v>
       </c>
@@ -12039,7 +12035,7 @@
       <c r="C222" s="21"/>
       <c r="D222" s="19"/>
     </row>
-    <row r="223" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="223" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A223" s="13">
         <v>44593</v>
       </c>
@@ -12049,7 +12045,7 @@
       <c r="C223" s="21"/>
       <c r="D223" s="19"/>
     </row>
-    <row r="224" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="224" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A224" s="13">
         <v>44621</v>
       </c>
@@ -12059,7 +12055,7 @@
       <c r="C224" s="21"/>
       <c r="D224" s="19"/>
     </row>
-    <row r="225" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="225" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A225" s="13">
         <v>44652</v>
       </c>
@@ -12069,7 +12065,7 @@
       <c r="C225" s="21"/>
       <c r="D225" s="19"/>
     </row>
-    <row r="226" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="226" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A226" s="13">
         <v>44682</v>
       </c>
@@ -12079,7 +12075,7 @@
       <c r="C226" s="21"/>
       <c r="D226" s="19"/>
     </row>
-    <row r="227" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="227" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A227" s="13">
         <v>44713</v>
       </c>
@@ -12089,7 +12085,7 @@
       <c r="C227" s="21"/>
       <c r="D227" s="19"/>
     </row>
-    <row r="228" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="228" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A228" s="13">
         <v>44743</v>
       </c>
@@ -12099,7 +12095,7 @@
       <c r="C228" s="21"/>
       <c r="D228" s="19"/>
     </row>
-    <row r="229" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="229" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A229" s="13">
         <v>44774</v>
       </c>
@@ -12109,7 +12105,7 @@
       <c r="C229" s="21"/>
       <c r="D229" s="19"/>
     </row>
-    <row r="230" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="230" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A230" s="13">
         <v>44805</v>
       </c>
@@ -12119,7 +12115,7 @@
       <c r="C230" s="21"/>
       <c r="D230" s="19"/>
     </row>
-    <row r="231" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="231" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A231" s="13">
         <v>44835</v>
       </c>
@@ -12129,7 +12125,7 @@
       <c r="C231" s="21"/>
       <c r="D231" s="19"/>
     </row>
-    <row r="232" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="232" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A232" s="13">
         <v>44866</v>
       </c>
@@ -12139,7 +12135,7 @@
       <c r="C232" s="21"/>
       <c r="D232" s="19"/>
     </row>
-    <row r="233" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="233" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A233" s="13">
         <v>44896</v>
       </c>
@@ -12149,7 +12145,7 @@
       <c r="C233" s="21"/>
       <c r="D233" s="19"/>
     </row>
-    <row r="234" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="234" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A234" s="13">
         <v>44927</v>
       </c>
@@ -12159,7 +12155,7 @@
       <c r="C234" s="21"/>
       <c r="D234" s="19"/>
     </row>
-    <row r="235" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="235" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A235" s="13">
         <v>44958</v>
       </c>
@@ -12169,7 +12165,7 @@
       <c r="C235" s="21"/>
       <c r="D235" s="19"/>
     </row>
-    <row r="236" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="236" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A236" s="13">
         <v>44986</v>
       </c>
@@ -12179,7 +12175,7 @@
       <c r="C236" s="21"/>
       <c r="D236" s="19"/>
     </row>
-    <row r="237" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="237" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A237" s="13">
         <v>45017</v>
       </c>
@@ -12189,7 +12185,7 @@
       <c r="C237" s="21"/>
       <c r="D237" s="19"/>
     </row>
-    <row r="238" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="238" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A238" s="13">
         <v>45047</v>
       </c>
@@ -12199,7 +12195,7 @@
       <c r="C238" s="21"/>
       <c r="D238" s="19"/>
     </row>
-    <row r="239" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="239" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A239" s="13">
         <v>45078</v>
       </c>
@@ -12209,7 +12205,7 @@
       <c r="C239" s="21"/>
       <c r="D239" s="19"/>
     </row>
-    <row r="240" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="240" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A240" s="13">
         <v>45108</v>
       </c>
@@ -12219,7 +12215,7 @@
       <c r="C240" s="21"/>
       <c r="D240" s="19"/>
     </row>
-    <row r="241" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="241" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A241" s="13">
         <v>45139</v>
       </c>
@@ -12229,7 +12225,7 @@
       <c r="C241" s="21"/>
       <c r="D241" s="19"/>
     </row>
-    <row r="242" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="242" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A242" s="13">
         <v>45170</v>
       </c>
@@ -12239,7 +12235,7 @@
       <c r="C242" s="21"/>
       <c r="D242" s="19"/>
     </row>
-    <row r="243" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="243" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A243" s="13">
         <v>45200</v>
       </c>
@@ -12249,7 +12245,7 @@
       <c r="C243" s="21"/>
       <c r="D243" s="19"/>
     </row>
-    <row r="244" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="244" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A244" s="13">
         <v>45231</v>
       </c>
@@ -12259,7 +12255,7 @@
       <c r="C244" s="21"/>
       <c r="D244" s="19"/>
     </row>
-    <row r="245" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="245" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A245" s="13">
         <v>45261</v>
       </c>
@@ -12269,7 +12265,7 @@
       <c r="C245" s="21"/>
       <c r="D245" s="19"/>
     </row>
-    <row r="246" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="246" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A246" s="13">
         <v>45292</v>
       </c>
@@ -12279,7 +12275,7 @@
       <c r="C246" s="21"/>
       <c r="D246" s="19"/>
     </row>
-    <row r="247" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="247" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A247" s="13">
         <v>45323</v>
       </c>
@@ -12289,7 +12285,7 @@
       <c r="C247" s="21"/>
       <c r="D247" s="19"/>
     </row>
-    <row r="248" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="248" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A248" s="13">
         <v>45352</v>
       </c>
@@ -12299,7 +12295,7 @@
       <c r="C248" s="21"/>
       <c r="D248" s="19"/>
     </row>
-    <row r="249" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="249" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A249" s="13">
         <v>45383</v>
       </c>
@@ -12309,7 +12305,7 @@
       <c r="C249" s="21"/>
       <c r="D249" s="19"/>
     </row>
-    <row r="250" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="250" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A250" s="13">
         <v>45413</v>
       </c>
@@ -12319,7 +12315,7 @@
       <c r="C250" s="21"/>
       <c r="D250" s="19"/>
     </row>
-    <row r="251" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="251" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A251" s="13">
         <v>45444</v>
       </c>
@@ -12329,7 +12325,7 @@
       <c r="C251" s="21"/>
       <c r="D251" s="19"/>
     </row>
-    <row r="252" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="252" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A252" s="13">
         <v>45474</v>
       </c>
@@ -12339,7 +12335,7 @@
       <c r="C252" s="21"/>
       <c r="D252" s="19"/>
     </row>
-    <row r="253" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="253" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A253" s="13">
         <v>45505</v>
       </c>
@@ -12349,7 +12345,7 @@
       <c r="C253" s="21"/>
       <c r="D253" s="19"/>
     </row>
-    <row r="254" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="254" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A254" s="13">
         <v>45536</v>
       </c>
@@ -12359,7 +12355,7 @@
       <c r="C254" s="21"/>
       <c r="D254" s="19"/>
     </row>
-    <row r="255" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="255" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A255" s="13">
         <v>45566</v>
       </c>
@@ -12369,7 +12365,7 @@
       <c r="C255" s="21"/>
       <c r="D255" s="19"/>
     </row>
-    <row r="256" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="256" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A256" s="13">
         <v>45597</v>
       </c>
@@ -12379,7 +12375,7 @@
       <c r="C256" s="21"/>
       <c r="D256" s="19"/>
     </row>
-    <row r="257" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="257" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A257" s="13">
         <v>45627</v>
       </c>
@@ -12389,7 +12385,7 @@
       <c r="C257" s="21"/>
       <c r="D257" s="19"/>
     </row>
-    <row r="258" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="258" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A258" s="13">
         <v>45658</v>
       </c>
@@ -12399,7 +12395,7 @@
       <c r="C258" s="21"/>
       <c r="D258" s="19"/>
     </row>
-    <row r="259" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="259" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A259" s="13">
         <v>45689</v>
       </c>
@@ -12409,7 +12405,7 @@
       <c r="C259" s="21"/>
       <c r="D259" s="19"/>
     </row>
-    <row r="260" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="260" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A260" s="13">
         <v>45717</v>
       </c>
@@ -12418,7 +12414,7 @@
       </c>
       <c r="D260" s="15"/>
     </row>
-    <row r="261" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="261" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A261" s="13">
         <v>45748</v>
       </c>
@@ -12427,7 +12423,7 @@
       </c>
       <c r="D261" s="15"/>
     </row>
-    <row r="262" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="262" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A262" s="13">
         <v>45778</v>
       </c>
@@ -12436,7 +12432,7 @@
       </c>
       <c r="D262" s="15"/>
     </row>
-    <row r="263" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="263" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A263" s="13">
         <v>45809</v>
       </c>
@@ -12445,112 +12441,112 @@
       </c>
       <c r="D263" s="15"/>
     </row>
-    <row r="264" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="264" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A264" s="13"/>
       <c r="B264" s="14"/>
       <c r="D264" s="15"/>
     </row>
-    <row r="265" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="265" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A265" s="13"/>
       <c r="B265" s="14"/>
       <c r="D265" s="15"/>
     </row>
-    <row r="266" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="266" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A266" s="13"/>
       <c r="B266" s="14"/>
       <c r="D266" s="15"/>
     </row>
-    <row r="267" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="267" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A267" s="13"/>
       <c r="B267" s="14"/>
       <c r="D267" s="15"/>
     </row>
-    <row r="268" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="268" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A268" s="13"/>
       <c r="B268" s="14"/>
       <c r="D268" s="15"/>
     </row>
-    <row r="269" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="269" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A269" s="13"/>
       <c r="B269" s="14"/>
       <c r="D269" s="15"/>
     </row>
-    <row r="270" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="270" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A270" s="13"/>
       <c r="B270" s="14"/>
       <c r="D270" s="15"/>
     </row>
-    <row r="271" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="271" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A271" s="13"/>
       <c r="B271" s="14"/>
       <c r="D271" s="15"/>
     </row>
-    <row r="272" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="272" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A272" s="13"/>
       <c r="B272" s="14"/>
       <c r="D272" s="15"/>
     </row>
-    <row r="273" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="273" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A273" s="13"/>
       <c r="B273" s="14"/>
       <c r="D273" s="15"/>
     </row>
-    <row r="274" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="274" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A274" s="13"/>
       <c r="B274" s="14"/>
       <c r="D274" s="15"/>
     </row>
-    <row r="275" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="275" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A275" s="13"/>
       <c r="B275" s="14"/>
       <c r="D275" s="15"/>
     </row>
-    <row r="276" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="276" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A276" s="13"/>
       <c r="B276" s="14"/>
       <c r="D276" s="15"/>
     </row>
-    <row r="277" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="277" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A277" s="13"/>
       <c r="B277" s="14"/>
       <c r="D277" s="15"/>
     </row>
-    <row r="278" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="278" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A278" s="13"/>
       <c r="B278" s="14"/>
       <c r="D278" s="15"/>
     </row>
-    <row r="279" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="279" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A279" s="13"/>
       <c r="B279" s="14"/>
       <c r="D279" s="15"/>
     </row>
-    <row r="280" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="280" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A280" s="13"/>
       <c r="B280" s="14"/>
       <c r="D280" s="15"/>
     </row>
-    <row r="281" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="281" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A281" s="13"/>
       <c r="B281" s="14"/>
       <c r="D281" s="15"/>
     </row>
-    <row r="282" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="282" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A282" s="13"/>
       <c r="B282" s="14"/>
       <c r="D282" s="15"/>
     </row>
-    <row r="283" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="283" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A283" s="13"/>
       <c r="B283" s="14"/>
       <c r="D283" s="15"/>
     </row>
-    <row r="284" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="284" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A284" s="13"/>
       <c r="B284" s="14"/>
       <c r="D284" s="15"/>
     </row>
-    <row r="285" spans="1:4" ht="17.25" x14ac:dyDescent="0.35">
+    <row r="285" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A285" s="16"/>
       <c r="B285" s="17"/>
       <c r="D285" s="15"/>

</xml_diff>